<commit_message>
Add department opening hours to HK private hospital haematology directory
- Rename service_hours to department_opening_hours with opening_hours_notes
- Add published clinic/lab hours for all 22 location rows
- Add Union Polyclinic TST and HKSH pathology lab rows
- Add department_opening_hours column to haematologists tab
- Regenerate Excel workbook and update README

Co-authored-by: jackiechow4567-arch <jackiechow4567-arch@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/industry/pm-reference/hk-private-hospitals-hematology.xlsx
+++ b/industry/pm-reference/hk-private-hospitals-hematology.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Haematologists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locations &amp; Contacts'!$A$1:$Q$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Haematologists'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locations &amp; Contacts'!$A$1:$Q$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Haematologists'!$A$1:$M$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -429,18 +429,18 @@
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="48" customWidth="1" min="13" max="13"/>
     <col width="48" customWidth="1" min="14" max="14"/>
     <col width="48" customWidth="1" min="15" max="15"/>
     <col width="48" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,25 +506,29 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>service_hours</t>
+          <t>department_opening_hours</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>opening_hours_notes</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>last_verified</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -586,15 +590,20 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Reception/clinic counter hours; haematology consultations by appointment within these hours</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Includes haematology nurse-led clinic; CAR-T and HSCT coordination</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/facilities-services/explore-facilities-and-services/specialist-outpatient-clinics/haematology-oncology-clinic</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -668,15 +677,20 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>Consultation by appointment only</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Adult haematology and cellular therapy; part of Comprehensive Oncology Centre network</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>https://www.hksh-hospital.com/en/hospital-directory</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -750,15 +764,20 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Oncology centre contact also used for haematology referrals at main campus</t>
+          <t>Same centre hours as adult haematology at Happy Valley</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>Oncology centre contact also used for paediatric haematology referrals at main campus</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>https://www.hksh-hospital.com/en/hospital-directory</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -832,15 +851,20 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>Consultation by appointment only</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Licensed private hospital site; CAR-T indicated for selected indications</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>https://www.hksh-emc.com/en/our-services/haematology.php</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -914,15 +938,20 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Paediatric blood diseases; HSCT; same building/contact as adult haematology centre</t>
+          <t>Same building and hours as adult haematology centre at Island East</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>Paediatric blood diseases; HSCT; shared contact with adult haematology centre</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>https://hksh-healthcare.com/en/clinical-services/paediatric-haematology-and-oncology-centre.php</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -988,15 +1017,20 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>Haematology consultations by appointment within clinic hours</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>In-hospital haematology consultation; hospital main line +852 2608 3388</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>https://www.union.org/en/service-overview/specialty/oncology</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1062,15 +1096,20 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Satellite oncology/haematology consultation site; also medical therapy Unit 206-207 and radiotherapy B1</t>
+          <t>Medical therapy (Unit 206-207) and radiotherapy (B1) follow same centre hours</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>Satellite oncology/haematology consultation site</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>https://www.union.org/en/service-overview/specialty/oncology</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1079,7 +1118,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hong Kong Adventist Hospital – Stubbs Road</t>
+          <t>Union Hospital</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1089,7 +1128,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hong Kong Adventist Hospital – Stubbs Road</t>
+          <t>Union Hospital Polyclinic (Tsim Sha Tsui)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1099,52 +1138,57 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Oncology Clinic</t>
+          <t>Union Hospital Polyclinic (Haematology)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1/F</t>
+          <t>Unit 1802, 18/F, Mira Place Tower A</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>40 Stubbs Road, Hong Kong</t>
+          <t>132 Nathan Road, Tsim Sha Tsui, Kowloon</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Central &amp; Western</t>
+          <t>Yau Tsim Mong</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>+852 3651 8808</t>
+          <t>+852 2375 3323</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>+852 3651 8833</t>
-        </is>
-      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>tst@union.org</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>By appointment</t>
+          <t>Mon-Fri 09:00-18:30; Sat 09:00-15:00; Sun/PH closed</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Hospital main enquiries +852 3651 8888; initial consult fee HK$1,500 (reference)</t>
+          <t>Dr Chan Cheuk Hung holds sessions here; book via polyclinic or hospital hotline</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>https://www.hkah.org.hk/en/specialist-clinics/oncology-clinic/contact</t>
+          <t>Haematology listed as polyclinic specialty; alternate site to Tai Wai / H Zentre</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
+        <is>
+          <t>https://www.union.org/tst/polyclinics/en/</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1153,7 +1197,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hong Kong Adventist Hospital – Tsuen Wan</t>
+          <t>Hong Kong Adventist Hospital – Stubbs Road</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1163,7 +1207,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hong Kong Adventist Hospital – Tsuen Wan</t>
+          <t>Hong Kong Adventist Hospital – Stubbs Road</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1173,50 +1217,54 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Outpatient / Specialist booking (hospital-wide)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+          <t>Oncology Clinic</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1/F</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>40 Stubbs Road, Hong Kong</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>199 Tsuen King Circuit, Tsuen Wan, N.T.</t>
+          <t>Central &amp; Western</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Tsuen Wan</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>+852 2275 6888</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>+852 2275 6767</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
+          <t>+852 3651 8808</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>+852 3651 8833</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>+852 2275 6888</t>
+          <t>Mon-Fri 09:00-17:30; Sat/Sun/hospital holiday closed</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Sun-Fri 08:00-17:00 (hospital service hours; PH closed)</t>
+          <t>Oncology clinic reception hours; haematology by appointment</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Haematology &amp; Haematological Oncology listed; Dr Chan Chee Wun Joyce; book via hospital line</t>
+          <t>Hospital main enquiries +852 3651 8888; initial consult fee HK$1,500 (reference)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://www.twah.org.hk/en/find-a-doctor</t>
+          <t>https://www.hkah.org.hk/en/specialist-clinics/oncology-clinic/contact</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1228,17 +1276,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Adventist Health (network)</t>
+          <t>Hong Kong Adventist Hospital – Tsuen Wan</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Adventist Medical Center – Causeway Bay</t>
+          <t>Hong Kong Adventist Hospital – Tsuen Wan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1248,56 +1296,57 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Haematology &amp; Haematological Oncology clinic</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Room 2601, 26/F, Lee Garden Two</t>
-        </is>
-      </c>
+          <t>Outpatient / Specialist booking (hospital-wide)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>28 Yun Ping Road, Causeway Bay, Hong Kong</t>
+          <t>199 Tsuen King Circuit, Tsuen Wan, N.T.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Wan Chai</t>
+          <t>Tsuen Wan</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>+852 2782 2202</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>info@adventistmedical.hk</t>
-        </is>
-      </c>
+          <t>+852 2275 6888</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>+852 2275 6767</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>+852 6119 1217</t>
+          <t>+852 2275 6888</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>By appointment</t>
+          <t>Sun-Fri 08:00-17:00; Sat closed; PH closed</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Not a licensed private hospital; Adventist network outpatient centre</t>
+          <t>Hospital service hours; specialist haematology by appointment</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>https://adventistmedical.hk/en/specialties/haematology-haematological-oncology</t>
+          <t>Haematology &amp; Haematological Oncology listed; Dr Chan Chee Wun Joyce; book via hospital line</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
+        <is>
+          <t>https://www.twah.org.hk/en/contact-us</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1316,7 +1365,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Adventist Medical Center – Taikoo Place</t>
+          <t>Adventist Medical Center – Causeway Bay</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1331,22 +1380,22 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>19/F, Oxford House, Taikoo Place</t>
+          <t>Room 2601, 26/F, Lee Garden Two</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>979 King's Road, Quarry Bay, Hong Kong</t>
+          <t>28 Yun Ping Road, Causeway Bay, Hong Kong</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Eastern</t>
+          <t>Wan Chai</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>+852 2309 5000</t>
+          <t>+852 2782 2202</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1357,25 +1406,30 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>+852 9316 7110</t>
+          <t>+852 6119 1217</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>By appointment</t>
+          <t>Mon-Thu 09:00-18:00; Fri 09:00-17:30; Sat/Sun/PH closed</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
+          <t>Centre opening hours; consultations by appointment</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
           <t>Not a licensed private hospital; Adventist network outpatient centre</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>https://adventistmedical.hk/en/specialties/haematology-haematological-oncology</t>
-        </is>
-      </c>
       <c r="P12" t="inlineStr">
+        <is>
+          <t>https://adventistmedical.hk/en/contact-us</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1384,17 +1438,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CUHK Medical Centre</t>
+          <t>Adventist Health (network)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CUHK Medical Centre</t>
+          <t>Adventist Medical Center – Taikoo Place</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1404,46 +1458,58 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Haematology &amp; Haematological Oncology (specialty outpatient)</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+          <t>Haematology &amp; Haematological Oncology clinic</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>19/F, Oxford House, Taikoo Place</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>979 King's Road, Quarry Bay, Hong Kong</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>9 Chak Cheung Street, Sha Tin, N.T.</t>
+          <t>Eastern</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Sha Tin</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>+852 3946 6888</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
+          <t>+852 2309 5000</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>info@adventistmedical.hk</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>general@cuhkmc.hk</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+          <t>+852 9316 7110</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Mon-Thu 09:00-18:00; Fri 09:00-17:30; Sat/Sun/PH closed</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>By appointment</t>
+          <t>Centre opening hours; consultations by appointment</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>In-house haematologist listed (Dr Li Wa); use general enquiry for appointment routing</t>
+          <t>Not a licensed private hospital; Adventist network outpatient centre</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>https://www.cuhkmc.hk/clinical-specialties/haematology-and-haematological-oncology</t>
+          <t>https://adventistmedical.hk/en/contact-us</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1455,7 +1521,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Matilda International Hospital</t>
+          <t>CUHK Medical Centre</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1465,56 +1531,60 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Matilda International Hospital</t>
+          <t>CUHK Medical Centre</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Clinical Haematology (visiting specialist)</t>
+          <t>Clinical Haematology &amp; Haematological Oncology</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Specialist Outpatient (Haematology)</t>
+          <t>Haematology &amp; Haematological Oncology (Oncology Centre)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>9 Chak Cheung Street, Sha Tin, N.T.</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>41 Mount Kellett Road, The Peak, Hong Kong</t>
+          <t>Sha Tin</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Central &amp; Western</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>+852 2849 0111</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>info@matilda.org</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>+852 3946 6288</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>general@cuhkmc.hk</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Mon-Fri 09:00-18:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>By appointment</t>
+          <t>Oncology Centre office hours; Dr Li Wa clinic sessions vary (see oncology consultation schedule)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Haematology listed as specialty; e.g. Dr Herman Liu (Honorary Consultant); no dedicated haematology centre page found</t>
+          <t>In-house haematologist listed (Dr Li Wa); Oncology Centre booking +852 3946 6288</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>https://www.matilda.org/en/find-a-doctor</t>
+          <t>https://www.cuhkmc.hk/hospital-service/medical-centres-allied-health/oncology-centre/consultation-sessions</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1526,7 +1596,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Hong Kong Baptist Hospital</t>
+          <t>Matilda International Hospital</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1536,66 +1606,63 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hong Kong Baptist Hospital</t>
+          <t>Matilda International Hospital</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Laboratory Haematology only</t>
+          <t>Clinical Haematology (visiting specialist)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pathology Department (Haematology section)</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>LG2, Block D</t>
-        </is>
-      </c>
+          <t>Specialist Outpatient (Haematology)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>222 Waterloo Road, Kowloon Tong, Kowloon</t>
+          <t>41 Mount Kellett Road, The Peak, Hong Kong</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Sham Shui Po</t>
+          <t>Central &amp; Western</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>+852 2339 8921</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>+852 2337 1658</t>
-        </is>
-      </c>
+          <t>+852 2849 0111</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>info@hkbh.org.hk</t>
+          <t>info@matilda.org</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Mon-Fri (Haematology section per hospital schedule)</t>
+          <t>Mon-Fri 08:30-17:30; Sat 08:30-13:30; Sun/PH closed</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Diagnostic/lab haematology; not a dedicated clinical haematology clinic</t>
+          <t>Specialist outpatient consultation hours; haematology by appointment</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>https://www.hkbh.org.hk/services-overview/investigative-services/pathology-department/?lang=en</t>
+          <t>Haematology listed as specialty; e.g. Dr Herman Liu (Honorary Consultant)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
+        <is>
+          <t>https://www.matilda.org/en/our-location</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1614,7 +1681,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HKBH East Kowloon Medical Centre</t>
+          <t>Hong Kong Baptist Hospital</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1624,48 +1691,61 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Core Laboratory</t>
+          <t>Pathology Department (Haematology section)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>27/F</t>
+          <t>LG2, Block D</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>8 Yan Yip Street, Kwun Tong, Kowloon</t>
+          <t>222 Waterloo Road, Kowloon Tong, Kowloon</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Kwun Tong</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+          <t>Sham Shui Po</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>+852 2339 8921</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>+852 2337 1658</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>labek@hkbh.org.hk</t>
+          <t>info@hkbh.org.hk</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Mon-Sat 09:30-18:30; Sun/PH closed</t>
+          <t>Mon-Fri 08:00-22:00; Sat 22:00-08:00 (extended/on-call coverage)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>CBC/ESR etc.; samples may be referred to main hospital lab</t>
+          <t>Haematology shares Blood Bank section hours; Immunology/Chemical Pathology Mon-Fri 09:00-17:00</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>https://www.hkbh.org.hk/EKMC/en/centre/core-laboratory/</t>
+          <t>Diagnostic/lab haematology; not a dedicated clinical haematology clinic</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
+        <is>
+          <t>https://www.hkbh.org.hk/services-overview/investigative-services/pathology-department/?lang=en</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1674,7 +1754,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>St. Paul's Hospital</t>
+          <t>Hong Kong Baptist Hospital</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1684,7 +1764,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>St. Paul's Hospital</t>
+          <t>HKBH East Kowloon Medical Centre</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1694,52 +1774,53 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pathology Department – Clinical Haematology</t>
+          <t>Core Laboratory</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>6/F, Main Block</t>
+          <t>27/F</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2 Eastern Hospital Road, Causeway Bay, Hong Kong</t>
+          <t>8 Yan Yip Street, Kwun Tong, Kowloon</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Wan Chai</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>+852 2837 5226</t>
-        </is>
-      </c>
+          <t>Kwun Tong</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>enquiry@stpaul.org.hk</t>
+          <t>labek@hkbh.org.hk</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>24-hr CBC available (per hospital pathology page)</t>
+          <t>Mon-Sat 09:30-18:30; Sun/PH closed</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Lab/diagnostic haematology; oncology at separate Radiotherapy and Oncology Centre (LG3; +852 2830 8637)</t>
+          <t>Core laboratory counter hours</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>https://www.stpaul.org.hk/en/center-and-service/detail/pathology-department</t>
+          <t>CBC/ESR etc.; samples may be referred to main hospital lab</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
+        <is>
+          <t>https://www.hkbh.org.hk/EKMC/en/centre/core-laboratory/</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1748,7 +1829,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Canossa Hospital</t>
+          <t>St. Paul's Hospital</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1758,7 +1839,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Canossa Hospital</t>
+          <t>St. Paul's Hospital</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1768,40 +1849,57 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Clinical Laboratory (Haematology section)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>Pathology Department – Clinical Haematology</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6/F, Main Block</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1 Old Peak Road, Mid-Levels, Hong Kong</t>
+          <t>2 Eastern Hospital Road, Causeway Bay, Hong Kong</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Central &amp; Western</t>
+          <t>Wan Chai</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>+852 2522 2181</t>
+          <t>+852 2837 5226</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>enquiry@stpaul.org.hk</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Clinical pathology lab: 24/7; Histopathology Mon-Fri 08:00-18:00, Sat 08:00-13:00, Sun/PH closed</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>HOKLAS-accredited lab haematology; no dedicated clinical haematology department identified</t>
+          <t>24-hr CBC and coagulation testing available</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>https://www.canossahospital.org.hk/en/service/diagnostic_services/laboratory/</t>
+          <t>Lab/diagnostic haematology; oncology at separate Radiotherapy and Oncology Centre (LG3; +852 2830 8637)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
+        <is>
+          <t>https://www.stpaul.org.hk/en/center-and-service/detail/pathology-department</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1810,7 +1908,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Evangel Hospital</t>
+          <t>Canossa Hospital</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1820,7 +1918,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Evangel Hospital</t>
+          <t>Canossa Hospital</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1830,44 +1928,61 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Laboratory Department (Haematology and Serology)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>Clinical Laboratory (Haematology section)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>4/F, Block A</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>222 Waterloo Road, Kowloon Tong, Kowloon</t>
+          <t>1 Old Peak Road, Mid-Levels, Hong Kong</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Sham Shui Po</t>
+          <t>Central &amp; Western</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>+852 2760 3442</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>+852 5741 4933</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>+852 2825 5333</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>+852 2825 5689</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>lab@canossahospital.org.hk</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Not published on hospital website — contact lab to confirm</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Hospital main +852 2711 5222; lab haematology tests only</t>
+          <t>After-hours/out-of-hours surcharge may apply per hospital fee schedule</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>https://www.evangel.org.hk/images/charges/list_lab_blood.pdf</t>
+          <t>HOKLAS-accredited lab haematology; no dedicated clinical haematology department identified</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
+        <is>
+          <t>https://www.canossahospital.org.hk/en/service/diagnostic_services/laboratory/fees_and_charges/</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -1876,7 +1991,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>St. Teresa's Hospital</t>
+          <t>Evangel Hospital</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1886,7 +2001,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>St. Teresa's Hospital</t>
+          <t>Evangel Hospital</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1896,50 +2011,50 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Clinical Laboratory (Haematology)</t>
+          <t>Laboratory Department (Haematology and Serology)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>1/F, Main Block</t>
+          <t>222 Waterloo Road, Kowloon Tong, Kowloon</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>327 Prince Edward Road, Kowloon</t>
+          <t>Sham Shui Po</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Kowloon City</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>+852 2200 3110</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>+852 2200 3111</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+          <t>+852 2760 3442</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>+852 5741 4933</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Lab service daily 07:30-23:00; blood draw 08:30-20:00; on-call 23:00-07:30</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>24/7 laboratory service</t>
+          <t>Includes Sundays and public holidays for lab service</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Lab haematology; hospital main +852 2200 3111</t>
+          <t>Hospital main +852 2711 5222; lab haematology tests only</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>https://www.sth.org.hk/medical_service.asp?dept_code=EHL&amp;lang_code=en</t>
+          <t>https://evangel.org.hk/en/services/diagnostic/lab/lab_3/</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -1951,71 +2066,246 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>St. Teresa's Hospital</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>St. Teresa's Hospital</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Laboratory Haematology only</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory (Haematology)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1/F, Main Block</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>327 Prince Edward Road, Kowloon</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Kowloon City</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>+852 2200 3110</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>+852 2200 3111</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>24/7</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Covers haematology and blood bank among other lab disciplines</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Lab haematology; hospital main +852 2200 3111</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>https://www.sth.org.hk/medical_service.asp?dept_code=EHL&amp;lang_code=en</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Precious Blood Hospital</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Precious Blood Hospital (Caritas)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Laboratory Haematology only</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Clinical Pathology Laboratory</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>4/F</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
         <is>
           <t>113 Castle Peak Road, Sham Shui Po, Kowloon</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Sham Shui Po</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>+852 3971 9900</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>+852 3971 9937</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
         <is>
           <t>enquiry@pbh.hk</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>24/7 inpatient lab operation; outpatient blood draw typically Mon-Sun 09:00-20:00</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Confirm current specimen collection times with lab +852 3971 9937</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
         <is>
           <t>HOKLAS clinical pathology lab; no dedicated clinical haematology department identified on public site</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>https://www.pbh.hk/en/contact-us</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>https://www.pbh.hk/clinical-laboratory/</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hong Kong Sanatorium &amp; Hospital</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Hong Kong Sanatorium &amp; Hospital</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Laboratory / Pathology Haematology only</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Department of Pathology (Haematology testing)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1/F, Li Shu Fan Block</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2 Village Road, Happy Valley, Hong Kong</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Wan Chai</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>+852 2835 8790</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>+852 2892 7502</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>lab@hksh-hospital.com</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Contact department for specimen hours</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Pathology haematology for diagnostics; separate from clinical Haematology and Cellular Therapy Centre</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Clinical pathology/lab haematology at main hospital pathology department</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>https://www.hksh-hospital.com/en/hospital-directory</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q21"/>
+  <autoFilter ref="A1:Q23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2026,7 +2316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2040,7 +2330,8 @@
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="48" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2086,20 +2377,25 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>department_opening_hours</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>appointment_contact</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>last_verified</t>
         </is>
@@ -2148,20 +2444,25 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:00-18:00; Sat 08:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>+852 3153 9000 / WhatsApp +852 6452 3581</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Also listed at HKSH Happy Valley</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/facilities-services/explore-facilities-and-services/specialist-outpatient-clinics/haematology-oncology-clinic</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2210,16 +2511,21 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:00-18:00; Sat 08:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>+852 3153 9000 / WhatsApp +852 6452 3581</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/medical-specialties/haematology-haematological-oncology</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2268,20 +2574,25 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:00-18:00; Sat 08:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>+852 3153 9000 / WhatsApp +852 6452 3581</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Also Honorary Consultant at Matilda International Hospital</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/medical-specialties/haematology-haematological-oncology</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2330,20 +2641,25 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:00-18:00; Sat 08:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>+852 3153 9000 / WhatsApp +852 6452 3581</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Also practices at Adventist network (Stubbs Road / AMC)</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/medical-specialties/haematology-haematological-oncology</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2392,16 +2708,21 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:00-18:00; Sat 08:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>+852 3153 9000 / WhatsApp +852 6452 3581</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/medical-specialties/haematology-haematological-oncology</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2450,16 +2771,21 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:00-18:00; Sat 08:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>+852 3153 9000 / WhatsApp +852 6452 3581</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>https://gleneagles.hk/medical-specialties/haematology-haematological-oncology</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2508,16 +2834,21 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>Happy Valley: Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed | Island East: Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>+852 2835 8877 (HV) / +852 2917 1200 (Island East)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
         <is>
           <t>https://hksh-healthcare.com/en/our-doctors/haematology-and-cellular-therapy-centre.php</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2566,16 +2897,21 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>Happy Valley: Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed | Island East: Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>+852 2835 8877 (HV) / +852 2917 1200 (Island East)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
         <is>
           <t>https://hksh-healthcare.com/en/our-doctors/haematology-and-cellular-therapy-centre.php</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2624,20 +2960,25 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>+852 2835 8877</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Also Co-Director at Gleneagles HK</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>https://mobile.hksh.com/en/taxonomy/term/1186/all</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2686,16 +3027,21 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>+852 2917 1200</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
         <is>
           <t>https://hksh-healthcare.com/en/our-doctors/paediatric-haematology-and-oncology-centre.php</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2744,16 +3090,21 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>Happy Valley: Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed | Island East: Mon-Fri 09:00-17:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>+852 2835 8877 (HV) / +852 2917 1200 (Island East)</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
         <is>
           <t>https://mobile.hksh.com/en/doctors/alphabetically/ALL</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2802,20 +3153,25 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>Contact department for specimen hours</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>+852 2835 8790</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Pathology/lab haematology not clinical outpatient clinic</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>https://mobile.hksh.com/en/doctors/alphabetically/ALL</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2864,20 +3220,25 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>Contact department for specimen hours</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>+852 2835 8790</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Pathology/lab haematology not clinical outpatient clinic</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>https://mobile.hksh.com/en/doctors/alphabetically/ALL</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2926,16 +3287,21 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>Tai Wai: Mon-Sat 09:00-18:00; Sun/PH closed | H Zentre TST: Mon-Fri 09:00-18:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>+852 2608 3315 (Tai Wai) / +852 2159 6100 (TST)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
         <is>
           <t>https://www.union.org/en/doctors/dr-chan-man-hong</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -2984,20 +3350,25 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>Tai Wai: Mon-Sat 09:00-18:00; Sun/PH closed | TST Polyclinic: Mon-Fri 09:00-18:30; Sat 09:00-15:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>+852 2608 3315 (Tai Wai) / Polyclinic TST via hospital booking</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>+852 2608 3388 for general booking</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>https://www.union.org/en/doctors/dr-chan-cheuk-hung</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -3046,20 +3417,25 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>Mon-Fri 09:00-17:30; Sat/Sun/hospital holiday closed</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>+852 3651 8808 / WhatsApp +852 3651 8833</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Also at Adventist Medical Centre (Lee Gardens / Taikoo)</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>https://www.hkah.org.hk/en/find-a-doctor/dr-ma-shing-yan-lawrence</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -3108,16 +3484,21 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>Sun-Fri 08:00-17:00; Sat closed; PH closed</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>+852 2275 6888</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
         <is>
           <t>https://www.twah.org.hk/en/find-a-doctor</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -3166,20 +3547,25 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>Mon-Thu 09:00-18:00; Fri 09:00-17:30; Sat/Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>+852 2782 2202 (CB) / +852 2309 5000 (TP)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Network outpatient centres (not licensed hospitals)</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://adventistmedical.hk/en/specialties/haematology-haematological-oncology</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -3228,16 +3614,21 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>Mon-Fri 09:00-18:00; Sat 09:00-13:00; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>+852 3946 6888 / general@cuhkmc.hk</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
         <is>
           <t>https://www.cuhkmc.hk/clinical-specialties/haematology-and-haematological-oncology</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
@@ -3286,27 +3677,32 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>Mon-Fri 08:30-17:30; Sat 08:30-13:30; Sun/PH closed</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>+852 2849 0111 / info@matilda.org</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Visiting/honorary specialist; book via hospital specialist outpatient</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>https://www.matilda.org/en/find-a-doctor/dr-herman-liu-sung-yu</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:M21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add inpatient pharmacy addresses for all 14 licensed private hospitals
- New hk-private-hospitals-inpatient-pharmacy.csv with floor, address, hours, and contacts
- Third Excel tab: Inpatient Pharmacies (one row per licensed hospital)
- Update build script, README, and hospitals landscape index

Co-authored-by: jackiechow4567-arch <jackiechow4567-arch@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/industry/pm-reference/hk-private-hospitals-hematology.xlsx
+++ b/industry/pm-reference/hk-private-hospitals-hematology.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet name="Locations &amp; Contacts" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Haematologists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Inpatient Pharmacies" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locations &amp; Contacts'!$A$1:$Q$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Haematologists'!$A$1:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inpatient Pharmacies'!$A$1:$O$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3705,4 +3707,1147 @@
   <autoFilter ref="A1:M21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>hospital_group</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>licensed_private_hospital</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>site_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>hospital_campus_address_en</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>inpatient_pharmacy_department</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>inpatient_pharmacy_floor_location</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>inpatient_pharmacy_address_en</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>telephone</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>fax</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>pharmacy_hours</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>last_verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gleneagles Hospital Hong Kong</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gleneagles Hospital Hong Kong</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1 Nam Fung Path, Wong Chuk Hang, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Southern</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Pharmacy Department / Gleneagles Dispensary</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>G/F, Tower A (left side of Front Desk)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>G/F, Tower A, Gleneagles Hospital Hong Kong, 1 Nam Fung Path, Wong Chuk Hang, Hong Kong</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>+852 3153 9750</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>dispensary@gleneagles.hk</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Dispensary counter Mon-Fri 09:00-17:30 (public holidays closed); hospital pharmacy provides 24-hour inpatient services</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Inpatient medications are prepared by the hospital pharmacy department; ward/unit-dose dispensing. Public dispensary counter hours differ from 24-hour inpatient pharmacy coverage.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://gleneagles.hk/facilities-services/gleneagles-dispensary-hong-kong</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hong Kong Sanatorium &amp; Hospital</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hong Kong Sanatorium &amp; Hospital</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2 Village Road, Happy Valley, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Wan Chai</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>G/F, Li Shu Pui Block (adjacent to 24-hour Outpatient Service reception)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>G/F, Li Shu Pui Block, Hong Kong Sanatorium &amp; Hospital, 2 Village Road, Happy Valley, Hong Kong</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>+852 2835 8600</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>+852 2892 7506</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>opd@hksh-hospital.com</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>24-hour (via G/F pharmacy linked to 24-hour Outpatient Service)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Hospital pharmacy department serves inpatients and outpatients; discharge medicines collected at G/F pharmacy near main entrance.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>https://www.hksh-hospital.com/en/clinical-services/24-hour-outpatient-service</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HKSH Eastern Medical Centre</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>HKSH Eastern Medical Centre (Tsao Yin Kai Block)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3 A Kung Ngam Village Road, Shau Kei Wan, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Eastern</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pharmacy Department (inpatient campus)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Floor not published on public website</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3 A Kung Ngam Village Road, Shau Kei Wan, Hong Kong (HKSH Eastern Medical Centre, Tsao Yin Kai Block)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>+852 2917 1000</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>+852 2558 8622</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>hospital@hksh-emc.com</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Contact hospital for current inpatient pharmacy hours</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Licensed inpatient hospital site. No public walk-in pharmacy counter listed at Island East outpatient buildings; inpatient pharmacy services operate internally at Tsao Yin Kai Block. Admission office: 2/F, +852 2917 5030.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>https://www.hksh-emc.com/en/our-services/tsao-yin-kai-block.php</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Union Hospital</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Union Hospital (Tai Wai)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>18 Fu Kin Street, Tai Wai, New Territories</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sha Tin</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>G/F, Union Hospital Medical Centre</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>G/F, Union Hospital Medical Centre, 18 Fu Kin Street, Tai Wai, New Territories</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>+852 2608 3388</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>union@union.org</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>24 hours</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Central hospital pharmacy for inpatient and outpatient dispensing at main Tai Wai campus.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://www.union.org/en/service-overview/allied-health-services/pharmacy</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hong Kong Adventist Hospital – Stubbs Road</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hong Kong Adventist Hospital – Stubbs Road</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>40 Stubbs Road, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Central &amp; Western</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pharmacy Services</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>G/F, main hospital lobby</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Ground Floor, Hong Kong Adventist Hospital, 40 Stubbs Road, Hong Kong</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>+852 3651 8888</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Pharmacy supportive service 08:00-23:00; 24-hour urgent inpatient medication coverage</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Inpatient unit-dose dispensing with barcode medication administration across wards; bedside discharge counselling available.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>https://www.hkah.org.hk/en/ancillary-services/pharmacy-services/contact</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hong Kong Adventist Hospital – Tsuen Wan</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Hong Kong Adventist Hospital – Tsuen Wan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>199 Tsuen King Circuit, Tsuen Wan, N.T.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Tsuen Wan</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2/F, Main Tower</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2/F, Main Tower, Hong Kong Adventist Hospital – Tsuen Wan, 199 Tsuen King Circuit, Tsuen Wan, N.T.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>+852 2275 6688</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Contact hospital for current pharmacy counter hours</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Inpatient and outpatient pharmacy with unit-dose dispensing and barcode medication administration.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>https://www.twah.org.hk/en/ancillary-services/pharmacy-2</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CUHK Medical Centre</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CUHK Medical Centre</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9 Chak Cheung Street, Sha Tin, N.T.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sha Tin</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pharmacy Department (inpatient)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1/F Pharmacy</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1/F Pharmacy, CUHK Medical Centre, 9 Chak Cheung Street, Sha Tin, N.T.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>+852 3946 6888</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>general@cuhkmc.hk</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>24-hour hospital (contact pharmacy via hospital main line)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Inpatient medications use closed-loop unit-dose dispensing to wards. G/F Outpatient Pharmacy is a separate public counter for outpatient services.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://www.cuhkmc.hk/knowing-us/background</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Matilda International Hospital</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Matilda International Hospital</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>41 Mount Kellett Road, The Peak, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Central &amp; Western</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Floor not published on public website</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>41 Mount Kellett Road, The Peak, Hong Kong (Matilda International Hospital)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>+852 2849 1531</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>phar@matilda.org</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Contact pharmacy for current hours</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Hospital pharmacy serves inpatients; discharge medicines arranged via ward/pharmacy. Patient Service Centre at G/F lobby handles admission.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://www.matilda.org/en/contact</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Hong Kong Baptist Hospital</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hong Kong Baptist Hospital</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>222 Waterloo Road, Kowloon Tong, Kowloon</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sham Shui Po</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G/F (Block B) and G/F (Block E)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>G/F (Block B) and G/F (Block E), Hong Kong Baptist Hospital, 222 Waterloo Road, Kowloon Tong, Kowloon</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>+852 2339 8964</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>info@hkbh.org.hk</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Block B Mon-Fri 09:00-18:00, Sat 09:00-16:00, Sun/PH closed; Block E 24 hours</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Block E pharmacy provides 24-hour inpatient/outpatient dispensing; Block B serves outpatient daytime hours.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>https://www.hkbh.org.hk/services-overview/paramedical-services/pharmacy/?lang=en</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>St. Paul's Hospital</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>St. Paul's Hospital</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2 Eastern Hospital Road, Causeway Bay, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Wan Chai</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Inpatient Pharmacy</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1/F, Main Block</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1/F, Main Block, St. Paul's Hospital, 2 Eastern Hospital Road, Causeway Bay, Hong Kong</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>+852 2837 5232</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>enquiry@stpaul.org.hk</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Inpatient pharmacy Mon-Sat 08:00-23:00, Sun 08:00-17:00; outpatient pharmacy 24/7 on same floor after hours</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>After inpatient pharmacy closes, services continue at outpatient pharmacy (1/F Main Block).</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.stpaul.org.hk/en/center-and-service/detail/pharmacy</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Canossa Hospital</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Canossa Hospital</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1 Old Peak Road, Mid-Levels, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Central &amp; Western</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Floor not published on public website</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1 Old Peak Road, Mid-Levels, Hong Kong (Canossa Hospital)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>+852 2522 2181</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>+852 2840 1986</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>enquiry@canossahospital.org.hk</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>24 hours, 7 days</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Hospital pharmacy dispenses for inpatients and outpatients; floor location not listed on public website.</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://www.canossahospital.org.hk/en/service/diagnostic_services/pharmacy/</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Evangel Hospital</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Evangel Hospital</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>222 Argyle Street, Kowloon, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Kowloon City</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Floor not published on public website</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>222 Argyle Street, Kowloon, Hong Kong (Evangel Hospital)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>+852 2711 5222</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>info@evanhosp.org.hk</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Contact hospital for current pharmacy hours</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Inpatient and outpatient dispensing, cytotoxic reconstitution, and clinical pharmacy services; specific pharmacy floor not listed on public website.</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>https://www.evangel.org.hk/en/services/allied/pharmacy/introduction</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>St. Teresa's Hospital</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>St. Teresa's Hospital</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>327 Prince Edward Road, Kowloon, Hong Kong</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kowloon City</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Pharmacy</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>G/F, Main Block</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>G/F, Main Block, St. Teresa's Hospital, 327 Prince Edward Road, Kowloon, Hong Kong</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>+852 2200 3106</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>+852 2200 3111</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>pharmacy@sth.org.hk</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Contact pharmacy for current hours</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Listed in hospital departmental directory at G/F Main Block.</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>https://www.sth.org.hk/service_directory.asp?lang_code=en</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Precious Blood Hospital</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Precious Blood Hospital (Caritas)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>113 Castle Peak Road, Sham Shui Po, Kowloon</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sham Shui Po</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Pharmacy Department</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Floor not published on public website</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>113 Castle Peak Road, Sham Shui Po, Kowloon (Precious Blood Hospital)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>+852 3971 9900</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>+852 2728 4290</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>enquiry@pbh.hk</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Contact hospital for current pharmacy hours</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>On-site pharmacy dispenses for inpatients and outpatients; specific floor not listed on public website.</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>https://www.pbh.hk/en/contact-us/</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>